<commit_message>
Forms sync auto batch 8: 5000 files
</commit_message>
<xml_diff>
--- a/salesforce_forms/015_expense_reimbursement_form--salesforce_forms.xlsx
+++ b/salesforce_forms/015_expense_reimbursement_form--salesforce_forms.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -893,7 +893,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Submitted by</t>
+          <t>Submitted By Email</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -916,7 +916,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Submitted on</t>
+          <t>Submitted On Date</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -939,7 +939,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Approved by</t>
+          <t>Approved By Email</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Approved on</t>
+          <t>Approved On Date</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -985,7 +985,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Denied by</t>
+          <t>Denied By Email</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Denied on</t>
+          <t>Denied On Date</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1102,8 +1102,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'options':_[{'name':_'category1'},_{'name':_'category2'},_{'name':_'category3'}]}</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'options': [{'name': 'category1'}, {'name': 'category2'}, {'name': 'category3'}]}</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1148,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'name':_'category4'}</t>
+          <t>category4</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'name': 'category4'}</t>
+          <t>category4</t>
         </is>
       </c>
     </row>
@@ -1165,12 +1165,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{'options':_[{'name':_'approved'},_{'name':_'denied'},_{'name':_'pending'}]}</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'options': [{'name': 'approved'}, {'name': 'denied'}, {'name': 'pending'}]}</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{'name':_'pending'}</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{'name': 'pending'}</t>
+          <t>pending</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'options':_[{'name':_'car_expense'},_{'name':_'meal_expense'},_{'name':_'travel_expense'}]}</t>
+          <t>option_1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{'options': [{'name': 'car_expense'}, {'name': 'meal_expense'}, {'name': 'travel_expense'}]}</t>
+          <t>Option 1</t>
         </is>
       </c>
     </row>
@@ -1216,12 +1216,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{'name':_'other_expense'}</t>
+          <t>other_expense</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{'name': 'other_expense'}</t>
+          <t>other expense</t>
         </is>
       </c>
     </row>

</xml_diff>